<commit_message>
abc2: documentos ficticios mucho más largos + vibe coding (mini web-app por rubro con Lovable/Gemini Canvas)
- Excel (20-84 filas) y TXT (largos, multi-sección) por rubro.
- Bonus vibe coding en Módulo 4: system prompt de una mini web-app útil según el
  rubro + un clic a Lovable y a Gemini (Canvas).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/abc2/material/educacion-notas.xlsx
+++ b/public/abc2/material/educacion-notas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,12 +407,15 @@
         <v>Trabajo 1</v>
       </c>
       <c r="C1" t="str">
-        <v>Prueba</v>
+        <v>Prueba escrita</v>
       </c>
       <c r="D1" t="str">
         <v>Oral</v>
       </c>
       <c r="E1" t="str">
+        <v>Trabajo 2</v>
+      </c>
+      <c r="F1" t="str">
         <v>Promedio</v>
       </c>
     </row>
@@ -421,72 +424,404 @@
         <v>Pérez, A.</v>
       </c>
       <c r="B2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Gómez, L.</v>
+        <v>Gómez, B.</v>
       </c>
       <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
         <v>6</v>
       </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
       <c r="D3">
         <v>7</v>
       </c>
       <c r="E3">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="F3">
+        <v>6.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Díaz, M.</v>
+        <v>Díaz, C.</v>
       </c>
       <c r="B4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E4">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="F4">
+        <v>7.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Ruiz, S.</v>
+        <v>Ruiz, D.</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Torres, E.</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>7</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Vega, F.</v>
+      </c>
+      <c r="B7">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>9</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Núñez, G.</v>
+      </c>
+      <c r="B8">
+        <v>10</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
         <v>6</v>
       </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
+      <c r="F8">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>López, H.</v>
+      </c>
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9">
+        <v>4</v>
+      </c>
+      <c r="F9">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Sosa, I.</v>
+      </c>
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10">
+        <v>9</v>
+      </c>
+      <c r="F10">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Molina, J.</v>
+      </c>
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>6</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>7</v>
+      </c>
+      <c r="F11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Ríos, K.</v>
+      </c>
+      <c r="B12">
+        <v>7</v>
+      </c>
+      <c r="C12">
+        <v>9</v>
+      </c>
+      <c r="D12">
+        <v>7</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Castro, L.</v>
+      </c>
+      <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>9</v>
+      </c>
+      <c r="E13">
+        <v>10</v>
+      </c>
+      <c r="F13">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Ortiz, M.</v>
+      </c>
+      <c r="B14">
+        <v>9</v>
+      </c>
+      <c r="C14">
+        <v>7</v>
+      </c>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <v>8</v>
+      </c>
+      <c r="F14">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Silva, N.</v>
+      </c>
+      <c r="B15">
+        <v>10</v>
+      </c>
+      <c r="C15">
+        <v>10</v>
+      </c>
+      <c r="D15">
+        <v>7</v>
+      </c>
+      <c r="E15">
+        <v>6</v>
+      </c>
+      <c r="F15">
+        <v>8.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Romero, O.</v>
+      </c>
+      <c r="B16">
+        <v>4</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16">
+        <v>9</v>
+      </c>
+      <c r="E16">
+        <v>4</v>
+      </c>
+      <c r="F16">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Herrera, P.</v>
+      </c>
+      <c r="B17">
+        <v>5</v>
+      </c>
+      <c r="C17">
+        <v>8</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>9</v>
+      </c>
+      <c r="F17">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Medina, Q.</v>
+      </c>
+      <c r="B18">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+      <c r="D18">
+        <v>7</v>
+      </c>
+      <c r="E18">
+        <v>7</v>
+      </c>
+      <c r="F18">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Flores, R.</v>
+      </c>
+      <c r="B19">
+        <v>7</v>
+      </c>
+      <c r="C19">
+        <v>6</v>
+      </c>
+      <c r="D19">
+        <v>9</v>
+      </c>
+      <c r="E19">
+        <v>5</v>
+      </c>
+      <c r="F19">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Acosta, S.</v>
+      </c>
+      <c r="B20">
+        <v>8</v>
+      </c>
+      <c r="C20">
+        <v>9</v>
+      </c>
+      <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>10</v>
+      </c>
+      <c r="F20">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Benítez, T.</v>
+      </c>
+      <c r="B21">
+        <v>9</v>
+      </c>
+      <c r="C21">
+        <v>4</v>
+      </c>
+      <c r="D21">
+        <v>7</v>
+      </c>
+      <c r="E21">
+        <v>8</v>
+      </c>
+      <c r="F21">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>